<commit_message>
Fix output guardrail ordering bug, add SLO tracking, escalation persistence TODO
- tickets.py: run check_output() before updated_history is built in both
  /ticket and /ticket/stream, so redacted PII doesn't leak back into
  conversation_history on the next turn. /ticket previously never called
  check_output() at all.
- agent5_escalation.py: TODO noting escalation_package["team"] is never
  persisted to support_tickets.assigned_team, so live escalations don't
  appear on the manager /escalations dashboard.
- CLAUDE.md: track the above TODO in the Post-deploy row; SLO sheet update
  note.
- eval/classification_slo_results.json, eval/cost_slo_results.json: real
  eval run outputs (TSR, per-category/severity/routing accuracy, critical
  misclassification rate, guardrail pass rate, per-ticket cost by route)
  used to fill in FinalProgressTracker.xlsx Sheet2 with our actual 14 SLOs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diagrams and tracker/FinalProgressTracker.xlsx
+++ b/diagrams and tracker/FinalProgressTracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubh\python_projects\course_5\project-description-master\Project-2-Enterprise Software Support &amp; Resolution Intelligence System\diagrams and tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABF9E25-BBF4-4DD1-A8B3-28FDE7654993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD60212-6C36-404A-B8A0-A18C890BB857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,26 +26,16 @@
     <author>shubh</author>
   </authors>
   <commentList>
-    <comment ref="G26" authorId="0" shapeId="0" xr:uid="{363B8968-199B-47F3-A729-C58BF5D178EC}">
+    <comment ref="G26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>shubh:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>shubh:
 memory management uses langraph inbuilt checkpointing. MemorySaver saves the full TicketState in RAM after every node, keyed by thread_id.this enables multi turn conversation. The graph restored prior state on each new turn. The decsion of production is PostgresSaver which persists to out postgreSQL database so conversation survive server restarts</t>
         </r>
       </text>
@@ -55,7 +45,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="204">
+  <si>
+    <t>Enterprise Support Intelligence System — Sprint Progress Tracker</t>
+  </si>
   <si>
     <t>Project Start Date:</t>
   </si>
@@ -480,10 +473,7 @@
     <t>Planning, documentation, architecture, evaluation</t>
   </si>
   <si>
-    <t>Enterprise Support Intelligence System — Sprint Progress Tracker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLO metric </t>
+    <t>S.No</t>
   </si>
   <si>
     <t>Category</t>
@@ -498,154 +488,175 @@
     <t>Achieved Value</t>
   </si>
   <si>
-    <t>Latency</t>
-  </si>
-  <si>
-    <t>Accuracy</t>
-  </si>
-  <si>
-    <t>Recall</t>
-  </si>
-  <si>
-    <t>LLM as a judge</t>
-  </si>
-  <si>
-    <t>Task Succes Rate(TSR)</t>
+    <t>Task Success Rate (TSR)</t>
+  </si>
+  <si>
+    <t>Quality</t>
+  </si>
+  <si>
+    <t>Measures whether the system produced a correct outcome (category + severity + routing all match golden set)</t>
+  </si>
+  <si>
+    <t>&gt;=90%</t>
+  </si>
+  <si>
+    <t>88.46% (52/55 scored, run 2026-07-10)</t>
+  </si>
+  <si>
+    <t>Answer Groundedness / Faithfulness</t>
+  </si>
+  <si>
+    <t>Every claim in the response grounded in retrieved context (LLM-as-judge)</t>
+  </si>
+  <si>
+    <t>&gt;=95%</t>
+  </si>
+  <si>
+    <t>82.9% (eval/eval_results.json, pipeline run)</t>
   </si>
   <si>
     <t>SQL Correctness</t>
   </si>
   <si>
-    <t>Faithfulness</t>
+    <t>Parameterized query results match ground truth on the golden set</t>
+  </si>
+  <si>
+    <t>Not yet measured - no dedicated check implemented in eval.py</t>
+  </si>
+  <si>
+    <t>Answer Relevance</t>
+  </si>
+  <si>
+    <t>Response addresses the customer's actual question (LLM-as-judge)</t>
+  </si>
+  <si>
+    <t>&gt;=0.85</t>
+  </si>
+  <si>
+    <t>0.812 (eval/eval_results.json, pipeline run)</t>
+  </si>
+  <si>
+    <t>P95 Latency - Standard Routes</t>
+  </si>
+  <si>
+    <t>Speed</t>
+  </si>
+  <si>
+    <t>End-to-end latency for RAG/SQL/Hybrid routes</t>
+  </si>
+  <si>
+    <t>&lt;=5s</t>
+  </si>
+  <si>
+    <t>Not yet measured - requires eval/load_test.py against live server</t>
+  </si>
+  <si>
+    <t>P95 Latency - Multi-Agent Route</t>
+  </si>
+  <si>
+    <t>End-to-end latency for Multi-Agent (escalation) route</t>
+  </si>
+  <si>
+    <t>&lt;=10s</t>
+  </si>
+  <si>
+    <t>Retrieval Quality Recall@5</t>
+  </si>
+  <si>
+    <t>Retrieval</t>
+  </si>
+  <si>
+    <t>Proportion of relevant documents successfully retrieved in top 5</t>
+  </si>
+  <si>
+    <t>Not implemented - check_context_precision() raises NotImplementedError (future sprint)</t>
   </si>
   <si>
     <t>Source Attribution Rate</t>
   </si>
   <si>
+    <t>Responses cite retrieved evidence rather than hallucinating</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>70.0% (35/50 scored cases had citations, eval_results.json)</t>
+  </si>
+  <si>
     <t>Context Precision</t>
   </si>
   <si>
+    <t>Proportion of retrieved chunks that are actually relevant</t>
+  </si>
+  <si>
+    <t>&gt;=0.80</t>
+  </si>
+  <si>
+    <t>Not implemented - requires per-chunk relevance labels (future sprint)</t>
+  </si>
+  <si>
     <t>Critical Misclassification Rate</t>
   </si>
   <si>
-    <t>Escalation Recall(Human Handoff)</t>
-  </si>
-  <si>
-    <t>Unautorized Data Access(RBAC)</t>
-  </si>
-  <si>
-    <t>Guardrail effectivness</t>
-  </si>
-  <si>
-    <t>Answer Relevance</t>
-  </si>
-  <si>
-    <t>Query Routing Accuracy</t>
-  </si>
-  <si>
-    <t>Risk Classification Accuracy</t>
-  </si>
-  <si>
-    <t>Correctness</t>
-  </si>
-  <si>
-    <t>Usefullness</t>
-  </si>
-  <si>
-    <t>Quality</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>Completeness</t>
-  </si>
-  <si>
-    <t>LLM Confidence</t>
-  </si>
-  <si>
-    <t>Retrieval</t>
-  </si>
-  <si>
-    <t>Safety</t>
-  </si>
-  <si>
-    <t>Correctness of generated answers</t>
-  </si>
-  <si>
-    <t>Usefulness of the retrieved chunks and   generated output to the query</t>
-  </si>
-  <si>
-    <t>Quality of retrieved documents —   proportion that are relevant</t>
-  </si>
-  <si>
-    <t>End-to-end request latency from query   submission to response delivery</t>
-  </si>
-  <si>
-    <t>Overall correctness of the system’s   answers against ground truth</t>
-  </si>
-  <si>
-    <t>Completeness — proportion of relevant   documents successfully retrieved</t>
-  </si>
-  <si>
-    <t>LLM-as-judge confidence score   evaluating overall output quality</t>
-  </si>
-  <si>
-    <t>Measures whether the system produced a correct outcome</t>
-  </si>
-  <si>
-    <t>Measures whether parameterized query results match ground truth on the golden set</t>
-  </si>
-  <si>
-    <t>the system proves its answer is grounded in retrieved evidence rather than hallucination</t>
-  </si>
-  <si>
-    <t>Measures how often a Critical ticket is not classified as Critical (false negative</t>
-  </si>
-  <si>
-    <t>100% recall is the only acceptable target — missing a single mandatory escalation is a system failure, not a statistical outlier.</t>
-  </si>
-  <si>
-    <t>Any cross-customer data access is a data breach with regulatory and legal consequences</t>
-  </si>
-  <si>
-    <t>Measured against defined attack types</t>
-  </si>
-  <si>
-    <t>Queries are routed to the correct service or agent.</t>
-  </si>
-  <si>
-    <t>Correctly identifies and classifies risk levels</t>
-  </si>
-  <si>
-    <t>&gt;=80%</t>
-  </si>
-  <si>
-    <t>&gt;=75%</t>
-  </si>
-  <si>
-    <t>&gt;=70%</t>
-  </si>
-  <si>
-    <t>&lt;=2s</t>
-  </si>
-  <si>
-    <t>&gt;=85%</t>
-  </si>
-  <si>
-    <t>&gt;=90%</t>
-  </si>
-  <si>
-    <t>&gt;=95%</t>
+    <t>Safety &amp; Security</t>
+  </si>
+  <si>
+    <t>Rate at which a Critical ticket is NOT classified as Critical (false negative)</t>
   </si>
   <si>
     <t>&lt;3%</t>
   </si>
   <si>
+    <t>0.0% (0/8 Critical golden-set cases misclassified, run 2026-07-10)</t>
+  </si>
+  <si>
+    <t>Escalation Recall (8 mandatory scenarios)</t>
+  </si>
+  <si>
+    <t>100% recall required - missing one mandatory escalation is a system failure, not a statistical outlier</t>
+  </si>
+  <si>
+    <t>100% (eval/eval_results.json, pipeline run)</t>
+  </si>
+  <si>
+    <t>Unauthorized Data Access (RBAC)</t>
+  </si>
+  <si>
+    <t>Any cross-customer data access is a data breach with regulatory/legal consequences</t>
+  </si>
+  <si>
     <t>0 violations</t>
   </si>
   <si>
-    <t>S.No</t>
+    <t>Not yet measured - no automated RBAC eval run</t>
+  </si>
+  <si>
+    <t>Guardrail Effectiveness</t>
+  </si>
+  <si>
+    <t>% of adversarial test set (prompt injection, PII, policy violation) correctly blocked</t>
+  </si>
+  <si>
+    <t>100% (3/3 adversarial cases blocked, run 2026-07-10)</t>
+  </si>
+  <si>
+    <t>Cost Per Ticket</t>
+  </si>
+  <si>
+    <t>Cost &amp; Reliability</t>
+  </si>
+  <si>
+    <t>Average Azure OpenAI cost per ticket across all agent calls</t>
+  </si>
+  <si>
+    <t>&lt;=$0.05 avg, $0.15 cap</t>
+  </si>
+  <si>
+    <t>Avg $0.00105/ticket, max $0.00169 (0 hard-cap breaches, 51/52 scored, run 2026-07-10). By route: RAG $0.00072, SQL $0.00089, Hybrid $0.00129, Multi-Agent $0.00146.</t>
+  </si>
+  <si>
+    <t>SLO Metric</t>
   </si>
 </sst>
 </file>
@@ -657,7 +668,7 @@
     <numFmt numFmtId="165" formatCode="d\-mmm\-yy"/>
     <numFmt numFmtId="166" formatCode="d\-mmm"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -743,48 +754,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -800,6 +769,23 @@
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="32">
@@ -967,12 +953,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD6EAF8"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -989,8 +969,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -1034,25 +1020,156 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBDC3C7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBDC3C7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFBDC3C7"/>
       </left>
       <right style="thin">
         <color rgb="FFBDC3C7"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
       <top style="thin">
         <color rgb="FFBDC3C7"/>
       </top>
       <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
+      <top style="thin">
         <color rgb="FFBDC3C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBDC3C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE7E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE7E6E6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1167,54 +1284,394 @@
     <xf numFmtId="0" fontId="5" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="30" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="31" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="30" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="31" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="30" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="30" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Aptos"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFDFEFE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFE7E6E6"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFDFEFE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFE7E6E6"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFE7E6E6"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFDFEFE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFE7E6E6"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFE7E6E6"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Aptos"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFDFEFE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFE7E6E6"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFE7E6E6"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Aptos"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFDFEFE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFE7E6E6"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFE7E6E6"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD6EAF8"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFE7E6E6"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FFE7E6E6"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FFD9E2F3"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="10"/>
+        <name val="Aptos"/>
+      </font>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBDC3C7"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBDC3C7"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFBDC3C7"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFBDC3C7"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFBDC3C7"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBDC3C7"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBDC3C7"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBDC3C7"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1225,6 +1682,25 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D64F8E0C-9862-496B-A528-A3ABF85B1FEC}" name="SLO_Tracker" displayName="SLO_Tracker" ref="A1:F15" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:F15" xr:uid="{D64F8E0C-9862-496B-A528-A3ABF85B1FEC}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{277A43F1-6B0A-4A52-8096-8A235D9D1FB2}" name="S.No" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{605AEB4C-A466-4B0D-AFA6-06970D9A7D15}" name="SLO Metric" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{4275066C-50D0-4155-8509-96D888498893}" name="Category" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{74A98750-0D1B-403E-96C8-576A55D9062D}" name="Description" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{2497659C-744A-42B4-9B1F-294618CB37D1}" name="Expected Target" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{A855CDFD-B108-4028-AD1F-1D9377E0268F}" name="Achieved Value" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1438,7 +1914,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1447,9 +1923,9 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1460,9 +1936,9 @@
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1473,32 +1949,32 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="11">
         <v>46185</v>
@@ -1507,14 +1983,14 @@
         <v>0.5</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1524,14 +2000,14 @@
         <v>0.5</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="15"/>
       <c r="G6" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1541,14 +2017,14 @@
         <v>0.5</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="15"/>
       <c r="G7" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1558,14 +2034,14 @@
         <v>0.5</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1575,19 +2051,19 @@
         <v>0.5</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="11">
         <v>46186</v>
@@ -1596,14 +2072,14 @@
         <v>0.5</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1613,14 +2089,14 @@
         <v>0.5</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F11" s="15"/>
       <c r="G11" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1630,19 +2106,19 @@
         <v>0.5</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="11">
         <v>46187</v>
@@ -1651,31 +2127,31 @@
         <v>0.5</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F13" s="15"/>
       <c r="G13" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="17">
         <v>0.5</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="15"/>
       <c r="G14" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1685,14 +2161,14 @@
         <v>1.5</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1702,53 +2178,53 @@
         <v>0.5</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="17">
         <v>1</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="17">
         <v>0.5</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B19" s="11">
         <v>46192</v>
@@ -1757,14 +2233,14 @@
         <v>1</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1774,14 +2250,14 @@
         <v>1.5</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F20" s="15"/>
       <c r="G20" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1791,14 +2267,14 @@
         <v>1</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F21" s="15"/>
       <c r="G21" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1808,10 +2284,10 @@
         <v>0.5</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="E22" s="54" t="s">
         <v>49</v>
+      </c>
+      <c r="E22" s="42" t="s">
+        <v>50</v>
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="16"/>
@@ -1823,14 +2299,14 @@
         <v>0.5</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F23" s="15"/>
       <c r="G23" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1840,14 +2316,14 @@
         <v>0.5</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F24" s="15"/>
       <c r="G24" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1857,53 +2333,53 @@
         <v>0.5</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F25" s="15"/>
       <c r="G25" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="12">
         <v>1</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F26" s="15"/>
       <c r="G26" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14"/>
       <c r="B27" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" s="24">
         <v>11</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F27" s="14"/>
       <c r="G27" s="14"/>
     </row>
-    <row r="28" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B28" s="11">
         <v>46193</v>
@@ -1912,121 +2388,121 @@
         <v>1</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E28" s="26" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F28" s="15"/>
       <c r="G28" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="17">
         <v>0.5</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F29" s="15"/>
       <c r="G29" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="12">
         <v>1</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F30" s="15"/>
       <c r="G30" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="17">
         <v>0.5</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F31" s="15"/>
       <c r="G31" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="12">
         <v>0.5</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F32" s="15"/>
       <c r="G32" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="17">
         <v>0.5</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F33" s="15"/>
       <c r="G33" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="12">
         <v>0.5</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F34" s="15"/>
       <c r="G34" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B35" s="11">
         <v>46194</v>
@@ -2035,104 +2511,104 @@
         <v>1</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F35" s="15"/>
       <c r="G35" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="17">
         <v>0.5</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F36" s="15"/>
       <c r="G36" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="12">
         <v>1</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E37" s="28" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F37" s="15"/>
       <c r="G37" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="17">
         <v>1</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F38" s="15"/>
       <c r="G38" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="12">
         <v>1</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F39" s="15"/>
       <c r="G39" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="14"/>
       <c r="B40" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C40" s="24">
         <v>9</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E40" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F40" s="14"/>
       <c r="G40" s="14"/>
     </row>
-    <row r="41" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B41" s="11">
         <v>46199</v>
@@ -2141,87 +2617,87 @@
         <v>0.5</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F41" s="15"/>
       <c r="G41" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="17">
         <v>0.5</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F42" s="15"/>
       <c r="G42" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="12">
         <v>0.5</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F43" s="15"/>
       <c r="G43" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="17">
         <v>0.5</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E44" s="29" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F44" s="15"/>
       <c r="G44" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="12">
         <v>0.5</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E45" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F45" s="15"/>
       <c r="G45" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B46" s="11">
         <v>46200</v>
@@ -2230,51 +2706,51 @@
         <v>0.5</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="E46" s="55" t="s">
         <v>102</v>
+      </c>
+      <c r="E46" s="43" t="s">
+        <v>103</v>
       </c>
       <c r="F46" s="15"/>
       <c r="G46" s="16"/>
     </row>
-    <row r="47" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="17">
         <v>0.5</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E47" s="60" t="s">
         <v>104</v>
+      </c>
+      <c r="E47" s="46" t="s">
+        <v>105</v>
       </c>
       <c r="F47" s="15"/>
       <c r="G47" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
       <c r="C48" s="12">
         <v>0.5</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F48" s="15"/>
       <c r="G48" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B49" s="11">
         <v>46201</v>
@@ -2283,87 +2759,87 @@
         <v>1</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F49" s="15"/>
       <c r="G49" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
       <c r="C50" s="17">
         <v>0.5</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F50" s="15"/>
       <c r="G50" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
       <c r="C51" s="12">
         <v>0.5</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F51" s="15"/>
       <c r="G51" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
       <c r="C52" s="12">
         <v>0.5</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F52" s="15"/>
       <c r="G52" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="14"/>
       <c r="B53" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C53" s="24">
         <v>6</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E53" s="25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F53" s="14"/>
       <c r="G53" s="14"/>
     </row>
-    <row r="54" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B54" s="11">
         <v>46206</v>
@@ -2372,100 +2848,100 @@
         <v>1</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E54" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F54" s="15"/>
       <c r="G54" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="10"/>
       <c r="B55" s="10"/>
       <c r="C55" s="12">
         <v>0.5</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F55" s="15"/>
       <c r="G55" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="10"/>
       <c r="B56" s="10"/>
       <c r="C56" s="17">
         <v>0.5</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F56" s="15"/>
       <c r="G56" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
       <c r="C57" s="12">
         <v>0.5</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="E57" s="56" t="s">
         <v>126</v>
+      </c>
+      <c r="E57" s="44" t="s">
+        <v>127</v>
       </c>
       <c r="F57" s="15"/>
       <c r="G57" s="16"/>
     </row>
-    <row r="58" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
       <c r="B58" s="10"/>
       <c r="C58" s="12">
         <v>0.5</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="E58" s="57" t="s">
         <v>128</v>
+      </c>
+      <c r="E58" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="F58" s="15"/>
       <c r="G58" s="16"/>
     </row>
-    <row r="59" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
       <c r="B59" s="10"/>
       <c r="C59" s="12">
         <v>0.5</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E59" s="32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F59" s="15"/>
       <c r="G59" s="16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B60" s="34"/>
       <c r="C60" s="34"/>
@@ -2480,7 +2956,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="14"/>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
@@ -2489,9 +2965,9 @@
       <c r="F61" s="14"/>
       <c r="G61" s="14"/>
     </row>
-    <row r="62" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B62" s="36"/>
       <c r="C62" s="36"/>
@@ -2500,64 +2976,64 @@
       <c r="F62" s="36"/>
       <c r="G62" s="36"/>
     </row>
-    <row r="63" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="37" t="s">
-        <v>133</v>
-      </c>
-      <c r="B63" s="58" t="s">
         <v>134</v>
       </c>
-      <c r="C63" s="59"/>
-      <c r="D63" s="59"/>
-      <c r="E63" s="59"/>
+      <c r="B63" s="47" t="s">
+        <v>135</v>
+      </c>
+      <c r="C63" s="48"/>
+      <c r="D63" s="48"/>
+      <c r="E63" s="48"/>
       <c r="F63" s="38"/>
       <c r="G63" s="38"/>
     </row>
-    <row r="64" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="39" t="s">
-        <v>135</v>
-      </c>
-      <c r="B64" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
+      <c r="B64" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="C64" s="48"/>
+      <c r="D64" s="48"/>
+      <c r="E64" s="48"/>
       <c r="F64" s="38"/>
       <c r="G64" s="38"/>
     </row>
-    <row r="65" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="B65" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="C65" s="59"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
+      <c r="B65" s="47" t="s">
+        <v>139</v>
+      </c>
+      <c r="C65" s="48"/>
+      <c r="D65" s="48"/>
+      <c r="E65" s="48"/>
       <c r="F65" s="38"/>
       <c r="G65" s="38"/>
     </row>
-    <row r="66" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="41" t="s">
-        <v>139</v>
-      </c>
-      <c r="B66" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="C66" s="59"/>
-      <c r="D66" s="59"/>
-      <c r="E66" s="59"/>
+      <c r="B66" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C66" s="48"/>
+      <c r="D66" s="48"/>
+      <c r="E66" s="48"/>
       <c r="F66" s="38"/>
       <c r="G66" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B66:E66"/>
     <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B66:E66"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -2565,336 +3041,640 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B05806-BC2B-4E4B-818C-1B26580EE6D9}">
-  <dimension ref="A1:F18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.21875" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="50" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" style="51" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" style="51" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.109375" style="51" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" style="51" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.44140625" style="51" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+    <row r="1" spans="1:21" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="52" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="53" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="53" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="53" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="53" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" s="54" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A2" s="55">
+        <v>1</v>
+      </c>
+      <c r="B2" s="56" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" s="56" t="s">
+        <v>148</v>
+      </c>
+      <c r="D2" s="56" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="57" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" s="58" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+      <c r="S2" s="49"/>
+      <c r="T2" s="49"/>
+      <c r="U2" s="49"/>
+    </row>
+    <row r="3" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A3" s="59">
+        <v>2</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="60" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="61" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="49"/>
+      <c r="U3" s="49"/>
+    </row>
+    <row r="4" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A4" s="59">
+        <v>3</v>
+      </c>
+      <c r="B4" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>148</v>
+      </c>
+      <c r="D4" s="63" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="F4" s="65" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+      <c r="M4" s="49"/>
+      <c r="N4" s="49"/>
+      <c r="O4" s="49"/>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="49"/>
+      <c r="R4" s="49"/>
+      <c r="S4" s="49"/>
+      <c r="T4" s="49"/>
+      <c r="U4" s="49"/>
+    </row>
+    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="59">
+        <v>4</v>
+      </c>
+      <c r="B5" s="60" t="s">
+        <v>159</v>
+      </c>
+      <c r="C5" s="60" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="60" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" s="61" t="s">
+        <v>161</v>
+      </c>
+      <c r="F5" s="62" t="s">
+        <v>162</v>
+      </c>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="49"/>
+      <c r="M5" s="49"/>
+      <c r="N5" s="49"/>
+      <c r="O5" s="49"/>
+      <c r="P5" s="49"/>
+      <c r="Q5" s="49"/>
+      <c r="R5" s="49"/>
+      <c r="S5" s="49"/>
+      <c r="T5" s="49"/>
+      <c r="U5" s="49"/>
+    </row>
+    <row r="6" spans="1:21" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A6" s="59">
+        <v>5</v>
+      </c>
+      <c r="B6" s="63" t="s">
+        <v>163</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="65" t="s">
+        <v>167</v>
+      </c>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
+      <c r="N6" s="49"/>
+      <c r="O6" s="49"/>
+      <c r="P6" s="49"/>
+      <c r="Q6" s="49"/>
+      <c r="R6" s="49"/>
+      <c r="S6" s="49"/>
+      <c r="T6" s="49"/>
+      <c r="U6" s="49"/>
+    </row>
+    <row r="7" spans="1:21" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A7" s="59">
+        <v>6</v>
+      </c>
+      <c r="B7" s="60" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" s="60" t="s">
+        <v>169</v>
+      </c>
+      <c r="E7" s="61" t="s">
+        <v>170</v>
+      </c>
+      <c r="F7" s="62" t="s">
+        <v>167</v>
+      </c>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+      <c r="M7" s="49"/>
+      <c r="N7" s="49"/>
+      <c r="O7" s="49"/>
+      <c r="P7" s="49"/>
+      <c r="Q7" s="49"/>
+      <c r="R7" s="49"/>
+      <c r="S7" s="49"/>
+      <c r="T7" s="49"/>
+      <c r="U7" s="49"/>
+    </row>
+    <row r="8" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A8" s="59">
+        <v>7</v>
+      </c>
+      <c r="B8" s="63" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="64" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="65" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="49"/>
+      <c r="P8" s="49"/>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+      <c r="S8" s="49"/>
+      <c r="T8" s="49"/>
+      <c r="U8" s="49"/>
+    </row>
+    <row r="9" spans="1:21" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A9" s="59">
+        <v>8</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" s="60" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" s="61" t="s">
+        <v>177</v>
+      </c>
+      <c r="F9" s="62" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="49"/>
+      <c r="O9" s="49"/>
+      <c r="P9" s="49"/>
+      <c r="Q9" s="49"/>
+      <c r="R9" s="49"/>
+      <c r="S9" s="49"/>
+      <c r="T9" s="49"/>
+      <c r="U9" s="49"/>
+    </row>
+    <row r="10" spans="1:21" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A10" s="59">
+        <v>9</v>
+      </c>
+      <c r="B10" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>172</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="E10" s="64" t="s">
+        <v>181</v>
+      </c>
+      <c r="F10" s="65" t="s">
+        <v>182</v>
+      </c>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
+      <c r="Q10" s="49"/>
+      <c r="R10" s="49"/>
+      <c r="S10" s="49"/>
+      <c r="T10" s="49"/>
+      <c r="U10" s="49"/>
+    </row>
+    <row r="11" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A11" s="59">
+        <v>10</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>183</v>
+      </c>
+      <c r="C11" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="E11" s="66" t="s">
+        <v>186</v>
+      </c>
+      <c r="F11" s="62" t="s">
+        <v>187</v>
+      </c>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
+      <c r="M11" s="49"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="49"/>
+      <c r="P11" s="49"/>
+      <c r="Q11" s="49"/>
+      <c r="R11" s="49"/>
+      <c r="S11" s="49"/>
+      <c r="T11" s="49"/>
+      <c r="U11" s="49"/>
+    </row>
+    <row r="12" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A12" s="59">
+        <v>11</v>
+      </c>
+      <c r="B12" s="63" t="s">
+        <v>188</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="E12" s="64" t="s">
+        <v>177</v>
+      </c>
+      <c r="F12" s="65" t="s">
+        <v>190</v>
+      </c>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="49"/>
+      <c r="L12" s="49"/>
+      <c r="M12" s="49"/>
+      <c r="N12" s="49"/>
+      <c r="O12" s="49"/>
+      <c r="P12" s="49"/>
+      <c r="Q12" s="49"/>
+      <c r="R12" s="49"/>
+      <c r="S12" s="49"/>
+      <c r="T12" s="49"/>
+      <c r="U12" s="49"/>
+    </row>
+    <row r="13" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A13" s="59">
+        <v>12</v>
+      </c>
+      <c r="B13" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="E13" s="66" t="s">
+        <v>193</v>
+      </c>
+      <c r="F13" s="62" t="s">
+        <v>194</v>
+      </c>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="49"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="49"/>
+      <c r="O13" s="49"/>
+      <c r="P13" s="49"/>
+      <c r="Q13" s="49"/>
+      <c r="R13" s="49"/>
+      <c r="S13" s="49"/>
+      <c r="T13" s="49"/>
+      <c r="U13" s="49"/>
+    </row>
+    <row r="14" spans="1:21" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A14" s="59">
+        <v>13</v>
+      </c>
+      <c r="B14" s="63" t="s">
+        <v>195</v>
+      </c>
+      <c r="C14" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="D14" s="63" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="42" t="s">
-        <v>142</v>
-      </c>
-      <c r="C1" s="42" t="s">
-        <v>143</v>
-      </c>
-      <c r="D1" s="42" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="42" t="s">
-        <v>145</v>
-      </c>
-      <c r="F1" s="42" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="43"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
-      <c r="A3" s="44">
-        <v>1</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="C3" s="45" t="s">
-        <v>163</v>
-      </c>
-      <c r="D3" s="46" t="s">
-        <v>171</v>
-      </c>
-      <c r="E3" s="47" t="s">
-        <v>187</v>
-      </c>
-      <c r="F3" s="45"/>
-    </row>
-    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A4" s="44">
-        <v>2</v>
-      </c>
-      <c r="B4" s="48" t="s">
-        <v>160</v>
-      </c>
-      <c r="C4" s="48" t="s">
-        <v>164</v>
-      </c>
-      <c r="D4" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="E4" s="50" t="s">
-        <v>188</v>
-      </c>
-      <c r="F4" s="48"/>
-    </row>
-    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A5" s="44">
-        <v>3</v>
-      </c>
-      <c r="B5" s="45" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="D5" s="51" t="s">
-        <v>173</v>
-      </c>
-      <c r="E5" s="47" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="45"/>
-    </row>
-    <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A6" s="44">
-        <v>4</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="C6" s="48" t="s">
-        <v>166</v>
-      </c>
-      <c r="D6" s="49" t="s">
-        <v>174</v>
-      </c>
-      <c r="E6" s="50" t="s">
-        <v>190</v>
-      </c>
-      <c r="F6" s="48"/>
-    </row>
-    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A7" s="44">
-        <v>5</v>
-      </c>
-      <c r="B7" s="45" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="45" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" s="51" t="s">
-        <v>175</v>
-      </c>
-      <c r="E7" s="47" t="s">
-        <v>191</v>
-      </c>
-      <c r="F7" s="45"/>
-    </row>
-    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A8" s="44">
-        <v>6</v>
-      </c>
-      <c r="B8" s="52" t="s">
-        <v>149</v>
-      </c>
-      <c r="C8" s="48" t="s">
-        <v>167</v>
-      </c>
-      <c r="D8" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="E8" s="50" t="s">
-        <v>188</v>
-      </c>
-      <c r="F8" s="48"/>
-    </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A9" s="44">
-        <v>7</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="45" t="s">
-        <v>168</v>
-      </c>
-      <c r="D9" s="51" t="s">
+      <c r="E14" s="64" t="s">
         <v>177</v>
       </c>
-      <c r="E9" s="47" t="s">
-        <v>187</v>
-      </c>
-      <c r="F9" s="45"/>
-    </row>
-    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A10" s="44">
-        <v>8</v>
-      </c>
-      <c r="B10" s="48" t="s">
-        <v>151</v>
-      </c>
-      <c r="C10" s="48" t="s">
-        <v>165</v>
-      </c>
-      <c r="D10" s="49" t="s">
-        <v>178</v>
-      </c>
-      <c r="E10" s="50" t="s">
-        <v>192</v>
-      </c>
-      <c r="F10" s="48"/>
-    </row>
-    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A11" s="44">
-        <v>9</v>
-      </c>
-      <c r="B11" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="D11" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="E11" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="F11" s="45"/>
-    </row>
-    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A12" s="44">
-        <v>10</v>
-      </c>
-      <c r="B12" s="48" t="s">
-        <v>154</v>
-      </c>
-      <c r="C12" s="48" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="49" t="s">
-        <v>180</v>
-      </c>
-      <c r="E12" s="53">
-        <v>1</v>
-      </c>
-      <c r="F12" s="48"/>
-    </row>
-    <row r="13" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A13" s="44">
-        <v>11</v>
-      </c>
-      <c r="B13" s="45" t="s">
-        <v>156</v>
-      </c>
-      <c r="C13" s="45" t="s">
-        <v>170</v>
-      </c>
-      <c r="D13" s="51" t="s">
-        <v>181</v>
-      </c>
-      <c r="E13" s="47" t="s">
-        <v>194</v>
-      </c>
-      <c r="F13" s="45"/>
-    </row>
-    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.35">
-      <c r="A14" s="44">
-        <v>12</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>157</v>
-      </c>
-      <c r="C14" s="48" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="49" t="s">
-        <v>182</v>
-      </c>
-      <c r="E14" s="53">
-        <v>1</v>
-      </c>
-      <c r="F14" s="48"/>
-    </row>
-    <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.35">
-      <c r="A15" s="44">
-        <v>13</v>
-      </c>
-      <c r="B15" s="45" t="s">
-        <v>158</v>
-      </c>
-      <c r="C15" s="45" t="s">
-        <v>170</v>
-      </c>
-      <c r="D15" s="51" t="s">
-        <v>183</v>
-      </c>
-      <c r="E15" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F15" s="45"/>
-    </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A16" s="44">
+      <c r="F14" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
+      <c r="N14" s="49"/>
+      <c r="O14" s="49"/>
+      <c r="P14" s="49"/>
+      <c r="Q14" s="49"/>
+      <c r="R14" s="49"/>
+      <c r="S14" s="49"/>
+      <c r="T14" s="49"/>
+      <c r="U14" s="49"/>
+    </row>
+    <row r="15" spans="1:21" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="67">
         <v>14</v>
       </c>
-      <c r="B16" s="48" t="s">
-        <v>159</v>
-      </c>
-      <c r="C16" s="48" t="s">
-        <v>170</v>
-      </c>
-      <c r="D16" s="49" t="s">
-        <v>184</v>
-      </c>
-      <c r="E16" s="53">
-        <v>1</v>
-      </c>
-      <c r="F16" s="48"/>
-    </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A17" s="44">
-        <v>15</v>
-      </c>
-      <c r="B17" s="45" t="s">
-        <v>161</v>
-      </c>
-      <c r="C17" s="45" t="s">
-        <v>148</v>
-      </c>
-      <c r="D17" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="E17" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="F17" s="45"/>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.35">
-      <c r="A18" s="44">
-        <v>16</v>
-      </c>
-      <c r="B18" s="48" t="s">
-        <v>162</v>
-      </c>
-      <c r="C18" s="48" t="s">
-        <v>148</v>
-      </c>
-      <c r="D18" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="E18" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="F18" s="48"/>
+      <c r="B15" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="C15" s="68" t="s">
+        <v>199</v>
+      </c>
+      <c r="D15" s="68" t="s">
+        <v>200</v>
+      </c>
+      <c r="E15" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="F15" s="70" t="s">
+        <v>202</v>
+      </c>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
+      <c r="M15" s="49"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="49"/>
+      <c r="P15" s="49"/>
+      <c r="Q15" s="49"/>
+      <c r="R15" s="49"/>
+      <c r="S15" s="49"/>
+      <c r="T15" s="49"/>
+      <c r="U15" s="49"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="49"/>
+      <c r="S16" s="49"/>
+      <c r="T16" s="49"/>
+      <c r="U16" s="49"/>
+    </row>
+    <row r="17" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="49"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="49"/>
+      <c r="R17" s="49"/>
+      <c r="S17" s="49"/>
+      <c r="T17" s="49"/>
+      <c r="U17" s="49"/>
+    </row>
+    <row r="18" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="49"/>
+      <c r="N18" s="49"/>
+      <c r="O18" s="49"/>
+      <c r="P18" s="49"/>
+      <c r="Q18" s="49"/>
+      <c r="R18" s="49"/>
+      <c r="S18" s="49"/>
+      <c r="T18" s="49"/>
+      <c r="U18" s="49"/>
+    </row>
+    <row r="19" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G19" s="49"/>
+      <c r="H19" s="49"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="49"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="49"/>
+      <c r="P19" s="49"/>
+      <c r="Q19" s="49"/>
+      <c r="R19" s="49"/>
+      <c r="S19" s="49"/>
+      <c r="T19" s="49"/>
+      <c r="U19" s="49"/>
+    </row>
+    <row r="20" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="49"/>
+      <c r="M20" s="49"/>
+      <c r="N20" s="49"/>
+      <c r="O20" s="49"/>
+      <c r="P20" s="49"/>
+      <c r="Q20" s="49"/>
+      <c r="R20" s="49"/>
+      <c r="S20" s="49"/>
+      <c r="T20" s="49"/>
+      <c r="U20" s="49"/>
+    </row>
+    <row r="21" spans="7:21" x14ac:dyDescent="0.25">
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="49"/>
+      <c r="P21" s="49"/>
+      <c r="Q21" s="49"/>
+      <c r="R21" s="49"/>
+      <c r="S21" s="49"/>
+      <c r="T21" s="49"/>
+      <c r="U21" s="49"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F15">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>ISNUMBER(SEARCH("Not",F2))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>